<commit_message>
Update lith class associated elements
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/aashtoM145.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/aashtoM145.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dponti/Documents/GitHub/def/Codelist Excel Files and Conversion Templates to XML/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A94638DF-522B-F747-B652-CB0B7B1B93CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC7B23C-D096-E34E-BFC8-78F09B188ED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="19920" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="35840" windowHeight="19920" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DictionaryName" sheetId="3" r:id="rId1"/>
@@ -827,9 +827,6 @@
     <t>a-8</t>
   </si>
   <si>
-    <t>//diggs:Lithology/diggs:classificationCode</t>
-  </si>
-  <si>
     <t>Well-graded mixture of stone fragments or gravel, coarse sand, fine sand, and a nonplastic or feebly plastic soil binder.This subgroup includes those materials consisting predominantly of stone fragments or gravel, either with or without a well-graded binder of fine material.</t>
   </si>
   <si>
@@ -876,6 +873,9 @@
   </si>
   <si>
     <t>AASHTO M 145-91</t>
+  </si>
+  <si>
+    <t>//diggs:LithologyObservation//diggs:classificationCode</t>
   </si>
 </sst>
 </file>
@@ -1130,6 +1130,42 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <color auto="1"/>
       </font>
@@ -1227,42 +1263,6 @@
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium7"/>
   <extLst>
@@ -1281,6 +1281,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="DictionaryName"/>
@@ -1301,35 +1302,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DictionaryName" displayName="DictionaryName" ref="A1:E3" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:E3" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Start" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Dictionary ID" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DictionaryFile" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="DictionaryName" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H14" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Definitions" displayName="Definitions" ref="A1:H14" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="A1:H14" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="11">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Start" dataDxfId="18">
       <calculatedColumnFormula>IF(ISNA(VLOOKUP(B2,AssociatedElements!B$2:B2837,1,FALSE)),"Not used","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="10">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="ID" dataDxfId="17">
       <calculatedColumnFormula>SUBSTITUTE(SUBSTITUTE(LOWER([1]!Definitions[[#This Row],[Name]])," ","_"),"/","_")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Name" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="DataType" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="QuantityClass" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Authority" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Reference" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1674,10 +1675,10 @@
         <v>233</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>275</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>276</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>235</v>
@@ -1748,14 +1749,14 @@
         <v>236</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F2" s="15"/>
       <c r="G2" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>234</v>
@@ -1774,14 +1775,14 @@
         <v>237</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E3" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F3" s="15"/>
       <c r="G3" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>234</v>
@@ -1800,14 +1801,14 @@
         <v>238</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F4" s="15"/>
       <c r="G4" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>234</v>
@@ -1826,14 +1827,14 @@
         <v>239</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F5" s="15"/>
       <c r="G5" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>234</v>
@@ -1852,14 +1853,14 @@
         <v>240</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F6" s="15"/>
       <c r="G6" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>234</v>
@@ -1878,14 +1879,14 @@
         <v>241</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F7" s="15"/>
       <c r="G7" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>234</v>
@@ -1904,14 +1905,14 @@
         <v>242</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>234</v>
@@ -1930,14 +1931,14 @@
         <v>243</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F9" s="15"/>
       <c r="G9" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>234</v>
@@ -1956,14 +1957,14 @@
         <v>244</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="15"/>
       <c r="G10" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>234</v>
@@ -1982,14 +1983,14 @@
         <v>245</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F11" s="15"/>
       <c r="G11" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>234</v>
@@ -2008,14 +2009,14 @@
         <v>246</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F12" s="15"/>
       <c r="G12" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>234</v>
@@ -2034,14 +2035,14 @@
         <v>247</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F13" s="15"/>
       <c r="G13" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>234</v>
@@ -2060,14 +2061,14 @@
         <v>248</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F14" s="15"/>
       <c r="G14" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>234</v>
@@ -2118,7 +2119,7 @@
         <v>249</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2130,7 +2131,7 @@
         <v>250</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2142,7 +2143,7 @@
         <v>251</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2154,7 +2155,7 @@
         <v>252</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2166,7 +2167,7 @@
         <v>253</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2178,7 +2179,7 @@
         <v>254</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2190,7 +2191,7 @@
         <v>255</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2202,7 +2203,7 @@
         <v>256</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2214,7 +2215,7 @@
         <v>257</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2226,7 +2227,7 @@
         <v>258</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2238,7 +2239,7 @@
         <v>259</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2250,7 +2251,7 @@
         <v>260</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -2262,7 +2263,7 @@
         <v>261</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>